<commit_message>
feat: add 18 new recipes with listicle and multi-variant support, image assets, and affiliate links
</commit_message>
<xml_diff>
--- a/affiliate-products.xlsx
+++ b/affiliate-products.xlsx
@@ -11,17 +11,17 @@
     <sheet name="Products" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Instructions" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="159">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -327,6 +327,153 @@
   </si>
   <si>
     <t xml:space="preserve">6 High-Protein Lunch Boxes Meal Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Air fryer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/TurboBlaze-Premium-Ceramic-Coating-90%C2%B0-450%C2%B0F/dp/B0C33CHG99?crid=29K174U7RQHED&amp;dib=eyJ2IjoiMSJ9.JvIQTiQYIa-7vH5--3jg964Nf0p9WdZAK-1rFngdE1qGM52kKAeYw9Spp1PcLbq2qNDAfw3uEx2H6W-EFkqsdxLXGnACw1V8E1qj9ygR4ltV8I7ae4AVnWNULiWAQn0XzCG3wxdpH4V3GpRQyA_duvD4pgTzx87lPL7Bi3RZ_Zv8qmydNpS3h2S9xcyOTN3Q7L0NxnhsP1zMshbUKW9-389sbsvxO8ivjkVLFTywoNY.x8J6j-z5dUwMipVngmAM2ij0iXUm61IpGmkBkKphkoU&amp;dib_tag=se&amp;keywords=air%2Bfryer&amp;qid=1787294833&amp;sprefix=air%2Bfr%2Caps%2C587&amp;sr=8-4&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1201615d33fb8c566ab906e6a65cd11d&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Air Fryer Garlic Parmesan Fries, Crispy Air Fryer Chicken Wings, Crispy Air Fryer Salmon Bites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airtight containers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Rubbermaid-Brilliance-Airtight-Container-BPA-Free/dp/B0752ZJ5LF?crid=Z0F89GGNT4UY&amp;dib=eyJ2IjoiMSJ9.5MRpyVweaPJP07XGqOBD1wsdmjhYMozLz6iXZz6aQWKYymueUSn82sJng_h6kVUZXe2WRHNRJTeVmfKQtgDUTT9GUKFVhjtniql21svT65gOVYaRHD15jDuzJh44Odpsz4D_qXvisfcJdjlhSPtJ2QH9f4o_I9l9MKA81HbEsYlaKAPx_TJmO2dY4n4oh155BIg45OGtNH1ligNedn0njlf--CK9VfN5_HJDRq8ik-G61pzopxg2a9vuuTH3t-vVpZ21D3Kf78X10JCuxcrz1bKNUsQH0gZ8d_6ytiGhY_Y.f9Nd8K9YN_4AuKc3xiCT9lEmMtQ-1a8gKo0a8Dwtm0s&amp;dib_tag=se&amp;keywords=airtight%2Bcontainer&amp;qid=1787294895&amp;sprefix=airtight%2Bconta%2Caps%2C557&amp;sr=8-19&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1a4abfd6227ead40175359daf590e743&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 No-Bake Energy Balls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burger press</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Cuisinart-CISB-111-Smashed-Burger-Press/dp/B07SZFHKVZ?crid=1IINFDVVYUJDM&amp;dib=eyJ2IjoiMSJ9.2HjCnozck-eoA00aOrjZesor3pCxus5hokq_4DlRPX4EnP6X1qF_V1fGRoaDGLWugk2N3z5YgQ4Y90253AUxfGHNXo2fSBW7zGJin2tRRwy457b1uzXsD2C6PzznhUdcrbEMlJJHTznVIreGy6Q4JGk_w-c6P_YoffVoOa3Q9TQM7jFnCBQkCJtaleh4OfgrW2CrDB49-fcwocVvX7JffiVbTe4RUbmjQ1xHPLciGZ4.v-APOZeiC_xO-YKvTb-XZdOv-Tag0mK_VV_Af7E_LAI&amp;dib_tag=se&amp;keywords=burger%2Bpress&amp;qid=1787294991&amp;sprefix=burger%2Bpr%2Caps%2C532&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=b5cec603147e56eec4c3073c54a1a1f1&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crispy Smash Burgers with Special Sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrus squeezer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Elite-Gourmet-ETS623-Grapefruits-Stainless/dp/B0CK9HJ7S2?crid=1YIQ27RXITQET&amp;dib=eyJ2IjoiMSJ9.MpofArt3UHaOnw_l4i2df38sTpxWZ2mm06nPKPRR6OM2tjaJKIvl9z7PW9TMde0bcK2LitegnDPKYwl_I9BNQzMLS5GTN5vkyyySMpSPRuf-WaVd3aHJIhxMcUo8kwfCWS6WqbjnbAmp-n_dHNP78PgaSUo0E5RTbi2OkFthR-YdJWhIRHBJx1ooKQMAt2XShRtb09VpZ1uWKw2gpjELCaFIMQ2WsE5hP7z9oDgGNDeHgkaZ32RtFb4R-5_IVumTkWFi1jkzuQiInSM7nEL0GiChFPNvlPQtQv2FfT_NuMg.icwAVliH5Ko-4s-E3V8fmVP9v9JZa6gWGcrFzqHvL8c&amp;dib_tag=se&amp;keywords=citrus%2Bsqueezer&amp;qid=1787295033&amp;sprefix=citrus%2Bsquee%2Caps%2C589&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=263283c6248f72d5cc927a2ce4d403b4&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat Chipotle Guacamole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flexible spatula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/ChefAide-Silicone-Ergonomic-Resistant-Nonstick/dp/B0CHGFG64S?crid=2A0SVC5HLZVJ1&amp;dib=eyJ2IjoiMSJ9.-rDpl5_Q4Gx78sf1baalWfpcVTZ7P4zGKH2CIIZvnR423EnItEOMbYiaGhkNPGk3fgCdca9ZnGU_BGN7ly2ItFTK2iM6-uL_AmRvHg1wdBMK5a_H2wISQnSSJbaQ0XFlHW5zev5ToeM8ChQZ9z_YvG1SdDEux6qsbJZsK99s6ByZ65VFsUQS3rPlVU7ubp8odf9uDhya2YmttiYzhUsjbQLVlVdYV_L0xLQOZAGOaDO88KrZiI1GCxTwOG4uum4uLoHwPkyP6jcWcCMa2wOAyyOFCp9GAsUSEuH8TwnoFf0.2Ya68W0VD7Rb3p8-9x7Et4cNA8ZgnokckXwyHfi3c2w&amp;dib_tag=se&amp;keywords=flexible%2Bspatula&amp;qid=1787295074&amp;sprefix=flexible%2Bspa%2Caps%2C567&amp;sr=8-9&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=7ed999d8d8e27438d02797241c24afc6&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glass meal prep bowls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Containers-Airtight-Leak-Proof-Microwave-Dishwasher/dp/B0DPJXW27G?crid=1CWVOGTYQYQ8Y&amp;dib=eyJ2IjoiMSJ9.ybs2wvTHoEH1p_vOKWw5BqHKflEJSlHogAZnV8P9w0UlCVIcbCLyeUJgxs4O3DCch-qu2f1tlq4MSRY_DIvvG_PdUlDCRvqTzjPcfbRa5c0Yw4yftAloxYMFkeRQZmZsaKYMS5GAr64RkYG-_5k7yzLOlYrjC3y3YbdYH_oJcLR-f-Bnzla80vE2l_XxgHhikQRmw7vkv1oub1w1fRnUvb68lKrMar5s8EHBgEL9oLVZgwua7y37zqWQ5jJrNOt25QlV6YMUtD8_JoAPwEUfHKDWYAFshngyYm0tD7KObcs.-ZtLxlyrwuMbqoRkWwOJeGKQdIwSQeb-TH3H94Xqff8&amp;dib_tag=se&amp;keywords=glass%2Bmeal%2Bprep%2Bbowls&amp;qid=1787295119&amp;sprefix=glass%2Bmeal%2Bprep%2Bbowls%2Caps%2C575&amp;sr=8-17&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=caf1539ee1a93341975fa80c9507a3c0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Lazy Breakfast Ideas Under 5 Minutes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infuser water bottle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/UTEBIT-Infuser-Insulated-Camping-Outdoor/dp/B0BR8SK56M?crid=33E7HR6O2HEPS&amp;dib=eyJ2IjoiMSJ9.y0PuPqw2grQkyLWqPgX_mQYsZ6vgR29h7ATgfAICQ-4Eszad_vgAGq-QZdGodPpoqiFEbyX_yd8CW-kOGnalTRLMvQBo5_DMFNXM5Ex1F6ERPPD0V6jJox-PW8cb0AOFHVCD8-552s5cQPRpsk7V_vwIgP4gr7f1dhUhT8mhxGoFRRVfM7BqrLTZsoxqo7weDbRR6fbGflbxdDVnC5nesSNbGIlVyJYKD_3C-xMmt1NDKjmZS1Lwe7AEDU_w0-wVt-BVEohQg401otSAgLIRtw0IbvJVBlGrhNWwdroelsI._k7QkHSbFAj85G9ckqAbOnrxWY32L4s13URp_8VgYcs&amp;dib_tag=se&amp;keywords=infuser%2Bwater%2Bbottle&amp;qid=1787295196&amp;sprefix=infuser%2Bwater%2Bbott%2Caps%2C533&amp;sr=8-5&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=c02dfdc05b9ed8e0cc5d5ce1e4d89838&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 Detox Water Recipes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instant-read thermometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Thermometer-Cooking-BACKLIGHT-WATERPROOF-Temperature/dp/B00S93EQUK?crid=2V45R8BOOGT2&amp;dib=eyJ2IjoiMSJ9.8Ger4dMy4c3dRylJ0ztFU3EMn17qargrZcTgRn6jMofvVZEAm0qcJ_VRE-2yUvgB4kicBhPr6QahzAhlE7EE9jPOtHsl1f7yZ3Qb5xcHVJ7ZWr5LvdSVRs4didU44e4BGd-ksJU1vNB7ieK7_4OAfNKukB2U_dIzt1A9hzOhIxBjXTjRDGsUZbvg315ak52dce9iXOajFRd9szjVKAv3pPAVrkH5dLhEnAk8XoyOgJuQG6pKRD07iOjR0ioY_vq2EWvCCud2q1gRMFFopSiTg6VvAi8NTf4368O1XYdLQXc.dv3EBSg01A8M-FRJVdXg58QbiKduIEOoz2gmOzndzGs&amp;dib_tag=se&amp;keywords=instant+read+thermometer&amp;qid=1787295246&amp;sprefix=instant+read+thermo%2Caps%2C605&amp;sr=8-7&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=ccaf292f3bc1f53792e628b2f803223e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat Chick-fil-A Chicken Sandwich, Copycat Raising Cane's Chicken Tenders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large mixing bowl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/WEPSEN-Stainless-Kitchen-Measuring-Prepping/dp/B0CT2NWXX8?content-id=amzn1.sym.29113e31-4f10-4131-ad60-91d41893b2fc%3Aamzn1.sym.29113e31-4f10-4131-ad60-91d41893b2fc&amp;crid=2PGTJ1KK0JV9E&amp;cv_ct_cx=large%2Bmixing%2Bbowl&amp;keywords=large%2Bmixing%2Bbowl&amp;pd_rd_i=B0CT2NWXX8&amp;pd_rd_r=9195d263-901a-4a9d-92a3-5b5b3c93cbb7&amp;pd_rd_w=uIsjq&amp;pd_rd_wg=3C3Ql&amp;pf_rd_p=29113e31-4f10-4131-ad60-91d41893b2fc&amp;pf_rd_r=1MM32EDSCWCZG5X1TCPG&amp;qid=1787295282&amp;sbo=9ZOMT9Jm0JH%2Ft%2BWi68iDSA%3D%3D&amp;sprefix=large%2Bmixing%2Bbow%2Caps%2C553&amp;sr=1-3-f7d8a1b7-d68f-4a86-bfcb-111c62272989-spons&amp;aref=uR0PevFOnJ&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9zZWFyY2hfdGhlbWF0aWM&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=c5a096620ca09998f1199d8e01b134ab&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Air Fryer Garlic Parmesan Fries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mason jars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Ball-Mouth-Mason-mason-Bands/dp/B097HTTNF3?crid=3EQ9W7GFM88NE&amp;dib=eyJ2IjoiMSJ9.lqj6Tzyfa-gcoNR1ERjIOYDT4frKh5IBawXIFyXnuydFyQqclrZBgW3OTNVjx9O9j6aYm06mRCgqHP5uS0UH6WVLV-7T3ah1O7TrqB_QDGYK1beIAUa8OvRjn8mt7FQ0gmnOIephoHXFnBo3AfNOIkTuDLgex9-XiNZ7DSpeUcYS6ycTtw2ROA4AFA2P5mQLsWvRGkHCfrkVQBXpt2zuiCNyYgEFa8Ev_9iWmLcDwrgTc2y6E-OZYxfVJlaWxZsVxxMBtwJEwqPriFVN3NCXsF3v-4oJGQ9holnbFR2dvZ0.ecf5ioiuMD1yPkTKbtsDFgosao1gsILrA7Sdq4ge9cQ&amp;dib_tag=se&amp;keywords=mason%2Bjars&amp;qid=1787295330&amp;sprefix=mason%2Bja%2Caps%2C589&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=f9026d2a5d2910079203befae79daf54&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 Overnight Oat Flavors Meal Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meat mallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/KitchenAid-KO119OHOBA-Gourmet-Tenderizer-9-45-Inch/dp/B07Q2WVG1Z?crid=38F4NQV8WDJOD&amp;dib=eyJ2IjoiMSJ9.k8Nt-b8zXr54n7L4-B4CKXAYf1FWHcwCUdjEv52YlIB2qJ3rh0z_xF719kyUxBjrOu4iFdAOZuKtoKDJzrAt8p0TclHqxQljGXjmwvmKQ2PTY_dEGuyvOShPGAup3mF_RyY89ydXyQNg3wjPZwiOUMmsT436OrhtH1LAhklyjAHsaZZ3D1RVbybQug6AUz020lImdzHczmZ17Uj7yyswn4gL9LukFRsbrWqBoOKd1OkW39xsh_zukHMRGJ5KsZeR5HMx9LOOm2u4jwAp-abdCEQcO2PNW5xmWuE3B7EFp6w.TbAuD567rEFWoPt_9qCXm5fE7Us8xYEd8SgvekViDYY&amp;dib_tag=se&amp;keywords=meat%2Bmallet&amp;qid=1787295368&amp;sprefix=meat%2Bmallet%2Caps%2C555&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=d2a147638fa7aabdf0f4e00752440447&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat Chick-fil-A Chicken Sandwich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oven-safe skillet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Lodge-Skillet-Pre-Seasoned-Ready-Stove/dp/B00006JSUA?crid=3AZT7NZUHRXBD&amp;dib=eyJ2IjoiMSJ9.KAwBSzSJL8L5NQvLjg83Wg4GkPnKsr5AbNi7kiAMn7zzmOAiELpFOh_dQKvCaTamh0-ClyzLuBkeqrQOdOo1RzY_Tv8JmCIL7uVB2vIIIADAM-bmDuAZUN748UDBeJDLbQHTk8ZqKvoPJl7vjarAlt1nstLYQqgth4CpWPKKGEUAznf4I9eefj58hqV_IbUY3h440imhMzzfHrDyuK18i0NuQdicqVIjTSFABkhcv14ooNcsvgJwr-VqnEAnXOuQ3Ik3jIR3BnAODTY9VEktNxVMShEhLQG27ulnxeKH6V0.KWHN3bnxg6zo2lXz_5VWpd6XceMfXAqmNiu28FGp0v4&amp;dib_tag=se&amp;keywords=oven%2Bsafe%2Bskillet&amp;qid=1787295409&amp;sprefix=oven%2Bsafe%2Bskill%2Caps%2C581&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=5abda6359e88e1a32c81cde06bbb4b2f&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-Pan Marry Me Chicken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pastry brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/HOTEC-Silicone-Resistant-Marinades-Dishwasher/dp/B09JNRZHRT?crid=IHGMIQ13RZ2R&amp;dib=eyJ2IjoiMSJ9.9PjoV_tUr5meI1KqtWNrWerj8iQYjaQUGDa1Q5z_1bBUqLA5vNaKD0Cd6N0uSrjIHq70Nxh90KFbNejI-VdvVeHuTq5Xip673_usxYz7nGpa6TYUgA1lsxMlS7AxpXDayCJ7x11mCutpUs-gXkt3eWCixf8w87_urNTxy58d9UA9DyfUmnHu9kvAkkf6lyY4dUAvtEJxP9J1OHGNKA9OVWY4-5uCI5RJ7GjVGMOsMmbj6Y3tmIy_01yhW2fLzpaiV-3NAb86ogBESTe2JWh0w8hTEyF4Th3L7ePJPv9Zd4o.wCCOBz8XAme674vClvmAT7zvnG1Asr6iopICDPKNnNI&amp;dib_tag=se&amp;keywords=pastry%2Bbrush&amp;qid=1787295453&amp;sprefix=pastry%2Bbrush%2Caps%2C579&amp;sr=8-9&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1a7a90fc0085edb0f8ba1813f16049fe&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat Texas Roadhouse Rolls with Cinnamon Butter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small mason jars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/ComSaf-Mini-Mason-Jars-4oz/dp/B09YRC9SXW?crid=CVHMLQUIH3FS&amp;dib=eyJ2IjoiMSJ9.6_G97mRQ6FsY74JoSCi-A4aYxpMtF9d6g81RQJdwj6UT9NdkqRjc2gJwVwQWVfPvV8XRux1JP4y9kwqa2ADx1w6VjBJ23LxbqTO7k0Obn0ybegP8zUjw0PrqYTVVvUp2a0ajUcti5I5JWimD1GyBnRv4uJMWHlwXZAJpl9IXHK1-Uw0bUko3KophDmYCt_NYZfZfqGOPDWlFbLTq5FdxW8VlUD1iO2Ssc3teq5Rz11spwrkj3SEG1wAZo1a602wKdl3mDCRA4v75uRoRs_L_-8OWXwhwXW2uBf8VkFQFVNE.SuvHK5fSC7xzDx0Wfrah1wVW6ZxEsIbyOYL2BbmApUk&amp;dib_tag=se&amp;keywords=small%2Bmason%2Bjars&amp;qid=1787295494&amp;sprefix=small%2Bmason%2Bja%2Caps%2C592&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=6312b0bb70fc760ae595d1739f0611b0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat McDonald's Big Mac Sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small saucepan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Cuisinart-719-16-Classic-Stainless-Saucepan/dp/B00008CM69?crid=3MDFOTS2HUROE&amp;dib=eyJ2IjoiMSJ9.QAinwdsK-CYNbBOjPxE3HMPr4hxU2ZhD8wbPZ1y-jiCtW_J1TbyOKBy1uxlp56ycFrfLdtWIV8XgIxRd-MKRPrnUi-rvJ9Wtrsbg_9oaYcmdaQLbPX-3rH9Zzz1WKYrYovhgiJjcIEnaEzQsRXExt5aIpewu97jUtL0_fBXfvMl-vbBv77V6r6-ZI4BlnSWaxXQ2VOHWuSgE4Ph51XRTBxVeym_JZ9k0bJMHJG9XeC6FR8TFN3-t4Jpa157YCOU6CV3d4dwgrNrmovn4d0leB44Xiu7Ojs1Q-NKkmaRyCz8.r1s79ymMmqskg66Gaphq_82T-VW6qdruYBAsp9lKE9U&amp;dib_tag=se&amp;keywords=small%2Bsaucepan&amp;qid=1787295530&amp;sprefix=small%2Bsaucep%2Caps%2C551&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=03169d89cccb51075cc93718a03703b8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crispy Air Fryer Salmon Bites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small whisk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/NileHome-Stainless-Whisking-Blending-Stirring-3/dp/B08SWBRTRK?crid=2SJCTGODY5ZTU&amp;dib=eyJ2IjoiMSJ9.9CbAVoJJ-Ip6yMNfWgFmaof9D1Rwh3PRS-hkzkoUO9UXyEi9aGNZfLqk38yttMH_gIM_pMu8rsQ3OqTX7Cz7b_4kY7e8p3TFRtzWIdmG9GB1EMuudgmX2-6Ta309ttVykeG5Gs7dD7B1cCFczjB2aM2HR6_fsvADbLSDBsU_PvB2wwj2MrjPe0g8qylrB3SV8bM_Z0RbQucRWzTtDUz3DZeH53K1f2Jq0Dq8xjjOwhVwj_YVrBiuFUBM7ZGkhyRN9BJPZA57d_mS7IHrbq36EDPecT3TlnwC8W0N8q3-f_s.LVwHcWq_WHK8mpgK_WNOW6vzASnGRE_SIIWMAgo9bfU&amp;dib_tag=se&amp;keywords=small%2Bwhisk&amp;qid=1787295573&amp;sprefix=small%2Bwhis%2Caps%2C595&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=ee49d14fa45547d3cbcada6d43130b5e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tall glasses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Drinking-Water-Crystal-Highball-Glasses/dp/B0DBL3WXYW?crid=3SDY3XAS1V3MU&amp;dib=eyJ2IjoiMSJ9.BruIBv41Cv5aVUrTFtq9KMMI_9pmyL-lJexIBGaQIQ6Nnnn46SlOV83fWHS5y-GEcT8BmfmCVOK-AJG9y9EtoGoLnZYxLB47GqrClAXiGuZoWbai6TJrjVKdjh4zCS5Q7ApeIc2_pwyb9EEqb79JxPtoDfsM4J4mpq7JG_w7yHo6_zJQPGGJ376cBjmAgFDRqF6C8KaIK_a8tLNkKLkf9qIeEafSuXlaVSqzsDyL2qOZBSQvKE3CoGOuHL4ps249H73ucMKJOv2iIWfKMDg4zh86imqfoTp3A_IUZTtjON8.0fQIsdvGGjfSPxZoE1fo31xzH1LgOEqHuGeBZscqLSs&amp;dib_tag=se&amp;keywords=tall%2Bglasses&amp;qid=1787295615&amp;sprefix=tall%2Bglas%2Caps%2C554&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=0ae6d191a7d037f96e6bede877489fe2&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copycat Wendy's Frosty</t>
   </si>
   <si>
     <t xml:space="preserve">HOW TO USE THIS FILE</t>
@@ -360,9 +507,9 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="4">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -383,70 +530,21 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF999999"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2D6A4F"/>
-        <bgColor rgb="FF008080"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFE8E3DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFE8E3DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE8E3DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE8E3DC"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -475,36 +573,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -517,66 +591,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF2D6A4F"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFE8E3DC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF999999"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -663,17 +677,14 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -760,446 +771,446 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70.84"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="n">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="1" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1315,49 +1326,266 @@
         <v>101</v>
       </c>
     </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="#https://www.amazon.com/Kitchen-box-Electric-Portable-Lightweight/dp/B09BVCPSBT?crid=3VOOQHPRRAU14&amp;dib=eyJ2IjoiMSJ9.YzI6Nwe0e0LhSZli4AKYq9ha5K4UuyxJHg6PQaSiXE0CdW2_VC5sH2tGkg7dk1GT5_gucZMkpXzA15tm5y1tePjryh2OwPpnkcclbieFD9ZPCYoXAUw34QzacQ_IZ-KjS8ipksC0tQvPFjU5PEBQL77s4gRnRrx4aj1uO68DRa8VUFvBycxijoWKncm7bFjFHGStnl3gmIIBa9mPqNNzYo2BWpesSotrbX2Ubm7czZw.OUTTsjiW_gcIbLyzuuyLmDO4UXFC-jTkr3MrgIhsPkE&amp;dib_tag=se&amp;keywords=stand%2Bmixer&amp;qid=1786446369&amp;sprefix=stand%2Bmi%2Caps%2C529&amp;sr=8-1&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=e34c5531e4877052aed1a04dc78d60af&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C3" r:id="rId2" display="#https://www.amazon.com/NutriChef-3-Piece-Nonstick-Kitchen-Baking/dp/B089N57JGS?crid=KROAKD3A8R8P&amp;currency=USD&amp;dib=eyJ2IjoiMSJ9.vAfxlVdVZSbP4HWzB0GLHWtMXiBuatAgnBw-K4h8izmdpq-qe_YmMs6JI2xSiNNAzSrzZWTHeDQdJ_W6gHiFYRtYdLKMk8nD9L4S3mFbsc0iKQiaL1E-YkkkdUq-ud5gSUNWGx5QjD2POPnSCTTAl5O8e9ZmqUe3CQjpG5B8K1os_iXhzYBycWVqv6Wpe2mNzlNJOpVJuMq4k9ee3tRTHSV0RPBWs_dqmSeae9hsJTH5XEVavE1cptJYeybqSponW6anEaV1NxCgumcTlZ2_mJ7yMxxpEePsX1XTC7ZPCUo.3LIgX1O64l1RNuSQVU6AGlfuxTZWQApaGrgjQo5FI4Q&amp;dib_tag=se&amp;keywords=baking%2Bsheet&amp;qid=1786446452&amp;sprefix=baking%2Bsh%2Caps%2C539&amp;sr=8-4&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=0af115230d1cd60bddee9e579b5929ab&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C4" r:id="rId3" display="#https://www.amazon.com/Reynolds-Kitchens-Unbleached-Parchment-Paper/dp/B07PFYT8MC?crid=KROAKD3A8R8P&amp;currency=USD&amp;dib=eyJ2IjoiMSJ9.vAfxlVdVZSbP4HWzB0GLHWtMXiBuatAgnBw-K4h8izmdpq-qe_YmMs6JI2xSiNNAzSrzZWTHeDQdJ_W6gHiFYRtYdLKMk8nD9L4S3mFbsc0iKQiaL1E-YkkkdUq-ud5gSUNWGx5QjD2POPnSCTTAl5O8e9ZmqUe3CQjpG5B8K1os_iXhzYBycWVqv6Wpe2mNzlNJOpVJuMq4k9ee3tRTHSV0RPBWs_dqmSeae9hsJTH5XEVavE1cptJYeybqSponW6anEaV1NxCgumcTlZ2_mJ7yMxxpEePsX1XTC7ZPCUo.3LIgX1O64l1RNuSQVU6AGlfuxTZWQApaGrgjQo5FI4Q&amp;dib_tag=se&amp;keywords=baking%2Bsheet&amp;qid=1786446490&amp;sprefix=baking%2Bsh%2Caps%2C539&amp;sr=8-1&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=aa66ed18094e202ded3c9cf8a7f54b44&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C5" r:id="rId4" display="#https://www.amazon.com/JUNADAEL-Set-Tablespoon-Cupcake-Truffles/dp/B0DK6TSL13?crid=33L9LZ2RJTE1&amp;dib=eyJ2IjoiMSJ9.XFIFyMgrvrvsXi55f-BN0UoOsJiH34EwAn4jDhGc6CAZwWMvYrBR-OLbpxOpfWYSW8GmG-mz6XG1YdAvPV02lr6kHOygJopAfP0avrpuYcWd-vcBj_7ira1ipYFhqInmxegAOKRsmpP2uhOm8mHRQoDeXhjKpwxIVG5Vs_ZBUTktiSmJtqaM7G8lOFDg24RJX5WffeEFIC6qVVBqv7KY4snCQNnnJbEat8LICCjLvgC20pOGH_OUS07HhbChZxwImlCY6D-3PUKqbHTc0GbXa2fo1z3BDi7-56MdWLr-E8A.URZOQa25lrWMSD9m_Ab9GGFeg_pWgsivkO9FMQKv5D0&amp;dib_tag=se&amp;keywords=cooking+scoop&amp;qid=1786446518&amp;sprefix=cooking+scoo%2Caps%2C536&amp;sr=8-6&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=55bfaaf1f0a0f165158f98fcccaec5b4&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C6" r:id="rId5" display="#https://www.amazon.com/Riccle-Decorating-Reusable-Scrapers-Couplers/dp/B0CGNZ7BGR?crid=1OWVPW5L845L5&amp;dib=eyJ2IjoiMSJ9.r78_q4mBTfhCDTJ2la6UcjhQ4tfjEn5JrNzHaq5rvqTFaNtjIJDw3Uc5YFXQ7dbVMMJdOseQ52sMPSZ2zP9SFL206Ovfq6dpdvwKIp9ISV0H9DbiLJH-IVMRdSuXBMFEHuySHvWwAq6SFR8SNX1V4MKDdBAZDtY2ZBtCCO0Tr0Huf7KG2_-JFgE-IdotN_aKgM1iGB4dVsIrdt22zXpiBhfhuZqt4bw6psIZOhJvscwK1YWgFdgTQdmx2gOK7foKBXGcmLn5mhDLHPZWJmMCWykvvyfpB3bkpFMJNiCuq1k.hnaOp3yrYkJ73229GQvMnxEE4MZwSEvsSWpdqyVVjEY&amp;dib_tag=se&amp;keywords=piping%2Bbag&amp;qid=1786446552&amp;sprefix=piping%2Bbag%2Caps%2C523&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=b85c9c984d8fdd05142f7e261c737eb8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C7" r:id="rId6" display="#https://www.amazon.com/SENSARTE-Nonstick-Skillet-Induction-Healthy/dp/B0D9Q7D9VS?crid=1VNIHLRVLUXBI&amp;dib=eyJ2IjoiMSJ9.41vwpolDYRfCYNkU-05YrjknucAQBPWNzUmJ855cYR_MDAffgvnHWfOhrh0cCmifc9Z9aUOH-1_Ik8ctBIUY8vP1HU7_IbE_PeR4qzS98kYMcpZG3qYk9CxTFOn4IcyU-RIoe7urNO2f0vVSzSh9jC_p7EtvtOvEi8tIQP6uvN_kbjiqEmn1SnFVO7Z8fKZ_l20uXf2EN49xvEX9pm8L5qu3X4ZRch4lyvGCoLG5Bdt_PJdpcSkOF4SiPaqsWTru7HQOvlnF0-RP5N5jj325B4Z8kFUT3qYLezZneZN6B4E.0PyDvgpsUiOyM1dCEQ8XuUVpibDpIFyr1DbXuKwBM9A&amp;dib_tag=se&amp;keywords=large%2Bskillet&amp;qid=1786446621&amp;sprefix=large%2Bskil%2Caps%2C540&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=e4d4a6882e8485e3994c48e0ae0643af&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C8" r:id="rId7" display="#https://www.amazon.com/Nonstick-Cookware-Resistant-Utensils-Stirring/dp/B0FRFPQ3N5?crid=27NC175XIRFRC&amp;dib=eyJ2IjoiMSJ9.7kdWYj9yf38TGskuggIcECMVhiK5gHgqGJ5qYyC6-PunHqegJgw5HLvW6CpY9skDWZ7gKdJTtUGejjz2NUUfmqMl-ojXYE4f0alkGc5atdnDv9WMfrmOv07DchBBxbv1C8Xi6p7pH7A0fto57eMjc7ydJwMYxbNA7ix02rrM9-HYyrzOWHiWpgaIJNRl2o7I-v4LKhOsICtZd8zpGSpTIVeMy8eIJ2tXAGFhSi4p97kbJQFobVB-BzBzyMIVPWOy5rc9w00nfz_Y0f3Q5kiYmWJ5EGEqQIJAjHi2HLtyEfE.U2K3-f3lbDJAuTF3149LHsXE7t8FBc8JDy-BBO_gi-o&amp;dib_tag=se&amp;keywords=wooden+spoon&amp;qid=1786446658&amp;sprefix=wooden+spo%2Caps%2C532&amp;sr=8-6&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=cb48013bb64f0951dc932f4e9d035ba2&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C9" r:id="rId8" display="#https://www.amazon.com/Urbanstrive-Container-Professional-Stainless-Vegetables/dp/B0CLB61K3H?crid=5T9XJ4E0FHE0&amp;dib=eyJ2IjoiMSJ9.kwfRvkcK5dOjAWPHKnjNWsNOxkwv03nr9cHyOIXphEEdQ5H_uOLBnWBexpKJE9qFmfzNC64e1MOtoxSweyJ1Q0kuCkfHuJzhEVg_0vyXp5lt1VbRNUJmiLFb23OVYM9OgbWH3U3MBXvA2Oq3fkDRqvUXAc74BAS1iVxKFbHHgKCVSU6qbxZpJd14f1mhg_bLPTTprYkc3KReqy25qPwsy79AqUR5rB3G0-WMPg1wj_zc5pAuiEIKa9lHggeOYdUweNhstatAaRuYpxTq9gyn6ut8LTD5H2qZ-wPILlYbrWo.X356NehuTgNKpWUplDFW32yNvnLBPhuGKUfbFUwlUNM&amp;dib_tag=se&amp;keywords=grater&amp;qid=1786446719&amp;sprefix=gra%2Caps%2C543&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=2f151667e30c8ca23d674f239a5c3866&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C10" r:id="rId9" display="#https://www.amazon.com/Clay-Fire-Matcha-Handcrafted-Traditional/dp/B0FL2SM8XP?crid=IMZULE719TD4&amp;dib=eyJ2IjoiMSJ9.10DLFdNYEm3vv-gGWwUknnjFU3JoISizCj2UAcFws-udV8sR4L5lgcJLN0mg1ZbSsxaHuPEMfv85B3b1piFI7jILtu9zEKHdtfiQKSOSJ1QNmeCWMDxw8NAIYoaBjjJ7_yGZ8v2k7us59aUExljqZjcK-VrztEgSz7rP59M9p2ysn0odwmgsYcJnVLs8vJggx0wOFW3rjnOHk1vb8GlTUXpLbDYHi5YwYi4nNIs_YO8zjsnmzIqQ5pbVqcv54XJfWI_nZ-gVvCdfP6tRqHUrB6TDDrCP6YA7XIIn73GGaOk.a3jcnWWUCQZKrqD0Y75WLbPZ73nHugMGSpQdCbEQ-LI&amp;dib_tag=se&amp;keywords=matcha%2Bwhisk&amp;qid=1786446749&amp;sprefix=matcha%2Bwish%2Caps%2C529&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=de5d48b5ad631782f917d21b214fe202&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C11" r:id="rId10" display="#https://www.amazon.com/Drinking-Water-Crystal-Highball-Glasses/dp/B0DBL3WXYW?crid=3HCSZLG75G5IK&amp;dib=eyJ2IjoiMSJ9.pMnrB7TmD_ZKW1_Bb9PMpatMVi4GEO61lvanLpzZ_VKmp19fJ5Xz8W06E26ZUw0ueYP2_v8ZU4KMltrMehQvpM_wslK5Xb5s7k28QSJpnel6lUpVNAiE1Kbk5ha2lBs7I2x0yx0iIUpCICDcU3fF1K78jjnIxnM_wHdXMegNXa8EXeoyNv7--3fYupUoW2eTMvXJmKqmLDBK2ujRVr02PaYgp60gYDU2SVNSg9NWnEvFPA2WSBzGRBPyfCofhIEFXvRKrT0csgKoJqCoWDdGeWfsvYMfQNzsUY-CRnTDVo4.VtoO0iCRnKuMcOddS0uyxns9xCztkh3Lu4epJe7HTWg&amp;dib_tag=se&amp;keywords=tall%2Bglass&amp;qid=1786446781&amp;sprefix=tall%2Bgla%2Caps%2C509&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=3fba6e3b07e56624a952abbe49c7b384&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C12" r:id="rId11" display="#https://www.amazon.com/CAMATET-Matcha-Ceramic-Japanese-Ceremonial/dp/B0DRG3H3DF?crid=FAPJBCM6Z33M&amp;dib=eyJ2IjoiMSJ9.lfeefNB1tMjmYcwXVDsJRJYSpoemPhVa4UK-j2GJOwXwk8c5Po0uiosc8HeFABXX86WnZYiRdTWzHh7mSRHfO-ZRUXTaPWkY0WS42gw5JR9n5vI9zVCDnqCZpyqw045vxZ_2QhmfnGgBCyTQ3nCexkRugv2bRDABI_VyRu-zIuV8n8Pd4-c3-5tQWauuzzOVAc988A3nAPoIf4n64hPJiaR6tK6Pj_56afbevmALpNORU1p7D0w4naEfMgV20myFsa9-pZdoN2N5GsdOPGhNtZIuyKD23q7qIxU5S1qpxNM.DLBwVaV-y9vWy3ldFtDzOZ8ChyP21PARXn1vN1oJo9I&amp;dib_tag=se&amp;keywords=ceramic%2Bmatcha%2Bbowl&amp;qid=1786446874&amp;sprefix=ceramic%2Bmatcha%2Bbowl%2Caps%2C550&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=27a02cf091a815572f336b072ed629b8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C13" r:id="rId12" display="#https://www.amazon.com/Ohtomber-Cocktails-Stainless-Accessories-Bartending/dp/B0DDB3JWPV?crid=37WP5NUSL9MJO&amp;dib=eyJ2IjoiMSJ9.Ma9yEK4EkPe_06fd9AvfO4TGZ0C8rZiDeOatRKez0pCz6W4_lozBAK4scWry6tTRRoxyCGLGFeCPO6eK4T7sRkBCoK89aw8sNFg90pE0fC4zvj2KgRcSyCTPXk6gx5icarXyGQBW2EiIz8bfXrdKBP3CfOWCTSxeEqmQ0B7rg3OxJl0h6_ELH4YJ08MGbdhpUBK5t0Ar8BW8-7cPrvuakOP0mXNv-MMt-ACqKEry0WaWwJXkhVKvfPuVqIA3VWehUidAF8lwg62nxUr9wM2j4hcXjGkwHuRqV7o49BfrG0E.vsEPjTNBH2RdcKMkNSwHtxBXt9NuEUdn6_YfMaiGSOI&amp;dib_tag=se&amp;keywords=muddler&amp;qid=1786446901&amp;sprefix=mu%2Caps%2C572&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=0fce22d45b473338647ec3819e2e14db&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C14" r:id="rId13" display="#https://www.amazon.com/Ninja-Professional-Countertop-Technology-BL610/dp/B00NGV4506?ie=UTF8&amp;s=psc&amp;sprefix=high%2Bspeed%2Bblen%2Caps%2C555&amp;keywords=high%2Bspeed%2Bblender&amp;crid=8IR2ALTQODKI&amp;dib_tag=se&amp;ASIN=B00NGV4506&amp;dib=eyJ2IjoiMSJ9.Xu0NhznEvkQP1KciA8NZDHe-rcH3gsM2nSIES7KCwadI2ceVCIX2xZtj-RYvRmri4N2KK0G4Yz-NGYGAjj26-GigSttjuVFLXJRqq1-VEKvauISIsVuGlKiWtKof5--ZqLJT8S4wQYZDzjgQjQf0kwc4cA62ElgfvR6Uuuxo1FuN3hVet9WV23ARtae_riyIUeU9Cy_cDz915ivQ_82j2JanKFoHWwSYiTvqCNlaovI.rUDn_kfuVLyZcVc3142tOm--PwBLtIixpBfHMS4nRas&amp;qid=1786446937&amp;sr=8-4&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=657f8897039b81a712107ed361fa52bb&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C15" r:id="rId14" display="#https://www.amazon.com/KOMUEE-Containers-Airtight-Microwave-Dishwasher/dp/B08X4615SC?crid=1SI7CH1MHL917&amp;dib=eyJ2IjoiMSJ9.8qyHg9ea13NFeMeAxetKh2-iCquJjIF3xUQQKnQLCODbh1LdpRYsciUoPjiJpAnhQ4XjHUDTje0uQMp8bpnBRaLmGXuxq3HhMrSOltE2ksiEe897P1Pu1sRe_ul7_DvWZkR4DngjeEWLFVtNlde7cuGRMNjT7Wyzx19R-a_yEmqjCFor1bh46IbsL9JytYn3Orsu8gRilpEyRu4R9qqc-wsyfumxjP9nklEE2rU1e2jePPR82Wk2XCN0l5gon_GXX2Nq4bpVoJbg9DTr8U8c9d2r3BcZ5Bv8g4loR0tgkTQ.VN6M4Ui67AVlhvxhbdJdeRY0AITQhFSGX6iH9vY5Q30&amp;dib_tag=se&amp;keywords=meal%2Bprep%2Bcontainer&amp;qid=1786446973&amp;sprefix=meal%2Bprep%2Bconta%2Caps%2C530&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=d9d16b42a9579989b1b25b3f23146655&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C16" r:id="rId15" display="#https://www.amazon.com/SENSARTE-Nonstick-Frying-Pan-Skillet/dp/B086PHS2V8?crid=41DYZZYQRTY0&amp;dib=eyJ2IjoiMSJ9.5BmhUdF-5NPg_yEGuG3w4K-dMF7fq5L5LJcB_-1SEYiK4hmdgKW2WN2lBspwzibWObgmA_4gsQ6_h4Ko3N8WYaCTfgFcIapBkrxhmxdubuJ5ZQ0wUWaCVGDr9kEbzSzoQV-9ybmoTwydtKI9ocWUI8t_UXEjnihAg8Jn0A_tDsLjjFFJGxkHhyopzRo2CiUsZheHFu7hY-NLmAR6Ltrim98yatrTSCJiddfXbsjrGKfzotTv3-HtU2mjzCLuSNvdC3R5O4qs3TUC5fA2p1O0_jy_XEJCwE6-lC0qR42ImmI.A5uckZCE9B0ulhG0W6rEAcuIJCZMT38ZitCXcRi5EIM&amp;dib_tag=se&amp;keywords=non-stick%2Bpan&amp;qid=1786447015&amp;sprefix=non-stick%2Bpan%2Caps%2C578&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=3361412a3d1428a57a42edbbe94764d8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C17" r:id="rId16" display="#https://www.amazon.com/goodcook-Nonstick-Bakeware-Cookie-multicolor/dp/B0026RHI3M?crid=11T6U8UXGRNXW&amp;dib=eyJ2IjoiMSJ9.mOWte96yz1MSPL7uQHwiZohIvuW5M_CuAn_sEpQrmKvGV4higERf6l-NyM74PX6s2_hhuLynQ4SUxJHhLEXQIgepwrdthLoFk08HULcVg8oRGwqt-6qqCAP0lC-BEBRUVoUPIWmR7S50uUD0d4cb_4VkXV2tXVfRPkRXtlCRRSGha4hta-W3mTBH_A09kexA3M1LdpRfceMD8QmoPObPT1CVQq_J-55oXKUc6SvE8txrsedvfYCG-fa_Wf6xn6q3DijlA0Ibw3x3cbuLlud5PDy6LeqvpjW2s3qvq65G6wI.Qo7DKRi1yPTsnyKOX3vevtWMwU6yOYFzdvBFIyR5Gy8&amp;dib_tag=se&amp;keywords=sheet+pan&amp;qid=1786447054&amp;sprefix=sheet+pan%2Caps%2C536&amp;sr=8-7&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=bccb3723493045315abf9f7611f91358&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C18" r:id="rId17" display="#https://www.amazon.com/Enameled-Cast-Iron-Dutch-Oven/dp/B0DXJTNWJN?crid=TVDOLLRZIF64&amp;dib=eyJ2IjoiMSJ9.1RipCjRwp4yv3IHs4x1q8C_SHUqcsbpeDpcbdBo-2JLg8h8Hno0IxKy4bvHTMR7d5rNN7yBKHLfA7NBx2NJaHvT2Ohu22gWLSZTcPrdJi7rPdUCAiygwung_RUk4M7N7vTP8t8Ytq9H_w98foCBjki5oHks6EayOci6I-KuuEVa7ZpchUe73DELoH0QfT8TAUq-pS76fqb2QkqCQCs7coDQ0LJaVLqV6BuzAX2Ebv4-avC37i466OiHsmY0RjMuCSXMvgwGKoxeh-f3JKkGJLMczFSBFxs_ocWal1dEobMw.iFhJ4TmTPbbwvTMXmy0ScGA-yfQqoJu8OtBFyQVJgmc&amp;dib_tag=se&amp;keywords=dutch%2Boven&amp;qid=1786447085&amp;sprefix=dutch%2Bover%2Caps%2C528&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=9e4698f1f0941d03ddf58d171adcebf3&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C19" r:id="rId18" display="#https://www.amazon.com/Eddeas-Kitchen-Tongs-Ergonomic-Stainless/dp/B093C29J8H?crid=2O3IUHHQ2ZBO3&amp;dib=eyJ2IjoiMSJ9.LzTWU6VQGbhVSKvPiNqAZUD742_iq0Zw71RphuFg8d62G9M4bOcLti3NmPk9vQe4QMbQ8mnpC7UubO39EXQERwnnQkQpOlObtmdKJICt25D0iZu3lJ_NEk9Xo6sKtqJdzmOh0_fe4c3ufp9C5hJmY06cMXhWQr9AvDk6dR-P5K9cSLV8IiB1CIXa8-7vjl4nfK5-yQW5-6mQMwyAwO3mLLIkEBetmKHTmj4ICG-JxW74DtfvQ5ZQacSqrHTnGJZ7UhXB-JyYiM7nkl0UxdnIkLN86bluscJhtuaUMfaH69E._KGJWRi4sFbC4SYSDCO7DCyzVz8bFIu6aERrOcB2qRk&amp;dib_tag=se&amp;keywords=tongs&amp;qid=1786447119&amp;sprefix=tongs%2Caps%2C565&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=c256996751729f5a9ad1fddb53e493f9&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C20" r:id="rId19" display="#https://www.amazon.com/Urbanstrive-Container-Professional-Stainless-Vegetables/dp/B0CLB61K3H?crid=2IZNL1K0JQAJY&amp;dib=eyJ2IjoiMSJ9.41fLi6DmGTcTCg8EK1IjGbZThva4b3KFrUQH2xbMoOJRLXEt60YNfhyCIO6L94xFuICtoblN5n2Y2v3P6Er6LUbOphl511rz8Hk1_TkeRdVVwsjxD77Sm2KhP50bdXYNvVy3uh22jM4ZCn28E9EgjIqXfABE_RpQWVTIr235irddiQUXqIWhBskvpSsn_GwHkXfwvpCBylmRzUPn8IjBJbexVQ4qZNcdvauLD0plrrNUpxwgg0Xq6UFXk9ytXpuLZCxvy5K-HN-83Bf18V4ShSmGzXNijyd4is6r6TTP81U.NPQq-f8XTzahtne0WCJ7W_XhRcArl16dTM9hsi0AvHc&amp;dib_tag=se&amp;keywords=box%2Bgrater&amp;qid=1786447158&amp;sprefix=box%2Bgrat%2Caps%2C537&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=4f2816e78ec12c5b614042555c900951&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C21" r:id="rId20" display="#https://www.amazon.com/2PCS-Cooling-Racks-Cooking-Baking/dp/B0D4LX9Z3Q?crid=27T9H7MSGF0UF&amp;dib=eyJ2IjoiMSJ9.TSX0iCqNKWpdOXmVpsHgaXWNX-L9ntUwKehc0DlAW4VDadj8UxbAEGVYJHQPhZibHagqUFUxFX1ZO1plYeV0aqkhAOfZvOL4rrN4qrlgpTxkeJBFEHZZYXQB1UE5QPPGGNatW1DEoDIubCvOOj-dLtuF8GIvyEHXnz4q3SVg6asa5pX7ZdOu9nqijmDQb224D74vLwoJVLKbsdgHYMIWpSU0sDkrtoTK_BIYOB46XQcixwbneAmwIyMSeLCOQGQ8zXpE772qyi4FZP7MyaR2aS6Otv1EmIF-nzkjpooCERU.XW6QJ3rlqWUdgpnB9HWpY7-dEekAhNOkOWN0DftZe9Y&amp;dib_tag=se&amp;keywords=cooling%2Brack&amp;qid=1786447189&amp;sprefix=cooling%2Bra%2Caps%2C560&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1687f5e0a7f3ffdc360872f6e8d1baa3&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C22" r:id="rId21" display="#https://www.amazon.com/Lodge-Seasoned-Cast-Iron-Skillet/dp/B00006JSUB?crid=1Q2IGX18JIM6A&amp;dib=eyJ2IjoiMSJ9.yT7gVNTZD5mfojg5mkVUKjYoTydauk8BC_qudoyBJdrIXbEoEA-4QoRZ1i4EoTpo_ppOJFv8-9wuOoq3Quj0iyyuv42oA9hNRetNZZ42Hpv7UD4MpUKbKb7nz0ZXU30zuBjnNAiLaVEpH-dPcx6cfzJdY7WUfgdfBxKm4V1J7FEkJWoMoESmeogDd8JmURtFaYp5SbA0O2wljcJ_Qij4poy0rRtK8uzHgg3kAv6EK2tJ5tdtzfaqMTa3U65wLuEHd1d9Iw1heZGaTPYVdkPduZEGzg82MN3CTlKfiOo1eSA._YC9cUc3sNY_jkRUKCLzrbaXdmINXm-3vo9tgS7MqGU&amp;dib_tag=se&amp;keywords=cast%2Biron%2Bskillet&amp;qid=1786447222&amp;sprefix=cast%2Biron%2Bskill%2Caps%2C537&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=8e8dc5234c7c93838118dc11699177b1&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C23" r:id="rId22" display="#https://www.amazon.com/NileHome-Stainless-Whisking-Blending-Stirring-3/dp/B08SWBRTRK?crid=2CS8NT5VFRFG6&amp;dib=eyJ2IjoiMSJ9.vn1T1LMF_WslotWzDq-_xU7cEuW1IsKeJTBHLKoHwqECcn_ciIvEA34guwMHwi-9rA_udHVc06PB31Si7opmh_wTAYahnUcerKGUbR2oFn1PKhUUdaBU1cggN-teWkfG9NkY-snv9h3Nma4uJthBuinfYpK4SxY4Jk5FaS5ao6YsCMUqzEZJ9MHJog13oNwgnPYYQQRiOvAJcFT3U_H-_KHv99p6nmOssVk69_3PHJUpM29uR87H_1lp0q3VkmPIL3tDs8E0H625NhU_OeRTf7vn159LNj3QHSoozbz_tSI.tgvCrPnEBw-R1p7aWEHwA2Pn6b-7kTQN_Xw-uI3G_vE&amp;dib_tag=se&amp;keywords=whisk&amp;qid=1786447261&amp;sprefix=whis%2Caps%2C575&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=421beec0b247ae768b05025544fc957e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C24" r:id="rId23" display="#https://www.amazon.com/MCIRCO-Piece-Deep-Glass-Baking/dp/B087QZQX8V?crid=NLU2FS2SXQJN&amp;dib=eyJ2IjoiMSJ9.mlJVPdQdvrLBNeuwr50fm5sI2K9XfC38wsBM2ef-MBNvgF0BlpY8fsWFQSj8lLXQk_IKHD8MenzoTJ_y5UEANjnoueHt2VFQLbsrrxHykxcsYLZJrPRgXdUaxq3d72qvoYRTS2BO7suwQaHTqKyBpWCuQeN_ONvQeqDcAUf_8goJp0SygO13jKyjfXXjBRlPawu4IuzisENgLlM0welZ5WIeah0r3QxoQLPCi1wBkdZXj-hif2Tj_yQL8TVdat-TPZNRlNSoDEuXJ5ErB9LQw5OjRpV8zyWy7459tq28m6c.pQUM1WHLOIvTRpWpMUA7nG5v1og0Ts1JtmVJaEpsOvI&amp;dib_tag=se&amp;keywords=baking%2Bdish&amp;qid=1786447291&amp;sprefix=baking%2Bdish%2Caps%2C547&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=437a061191d42f80670369965f4c3ff0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C25" r:id="rId24" display="#https://www.amazon.com/SENSARTE-Nonstick-Stay-Cool-Induction-Compatible/dp/B0BJZCNYKG?crid=39VRGASZJMZKT&amp;dib=eyJ2IjoiMSJ9.YtPzn-yuW0t8dSo_qcnvellP3kNUAw57Bh2Vdav0OyfASWbMzB8Mlyi346Ad1PzdkaFocrehT_i-jVmso-TnnWHTMKHQQ-uMTiRDpk8_VH0vVW-4nrTSnsChMB3HER3MEn4XEkRlic8XEtaPxittBFsxRcmBbKZzzjHXLf3V3mfKeIfMdUsCiaTvOGKpTtFlDIC2fPWMB3P0tbd56SeAT94fqwJPU9G36XrpvGioprEljQ1E3B3DIthIalW-uLvVjMpzE7LYNWgUUdzEWjcBJiFq5Ml9oTLCmwh35Z7rNbk.nUyYcv27hFAEN6viD8AGb0Jzgm09oImB9lPDJnge80M&amp;dib_tag=se&amp;keywords=non-stick%2Bgriddle&amp;qid=1786447330&amp;sprefix=non-stick%2Bgrid%2Caps%2C591&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=935a2b6c3840313a586a068d42fd5423&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C26" r:id="rId25" display="#https://www.amazon.com/Umite-Chef-Airtight-Stainless-Attachments/dp/B0CGWQ53L3?crid=23ZP398JASWMB&amp;dib=eyJ2IjoiMSJ9.XvYIKVs6ZhMBJ7V3gogPAQugzzPma9lm5nRm2D0vJrOevLp9aZ3FlgL_oN7yDr-NCY1wE71n-FVBqB4_3aJOGVaVuonJdd7fKONmS-ZahgY9w5_EYU5YAAtael6OPgyVzhDvFvOLKqrqpytpTpNmSMy5NaqAcxvVIvZ6fH5kzeC-aCI17x_Y8CyKhjHws6NkFGLrqYWJ3iOLZTWVIID9b-BJBDOXGN_0j2X9J3DXeTUcjcWVB6l8yOVG5jelDiG_ayx5cckAcckF8fvv0Wt5hy__mP9TRfXazX7cqcr32kU.skLDbAV0BgyUNWIjijtXKeSrUL_W09M3IfGWTTrl3Z0&amp;dib_tag=se&amp;keywords=mixing%2Bbowl&amp;qid=1786447369&amp;sprefix=mixing%2Bbow%2Caps%2C594&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=15877a9b938b4abb43ad08aa4a9abef1&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C27" r:id="rId26" display="#https://www.amazon.com/Zulay-Inch-Stainless-Steel-Ladle/dp/B07QMZ5JJH?crid=3G6PGLFSHS69L&amp;dib=eyJ2IjoiMSJ9.Aw-TAYMd_cWyqjQKntFWlVknrTE-dFbXIDpRwV42ByZNdOVaQOWMU74-vgJBuXe21Q14eGpkoHAUmqSf5IZdpCG8t-uW6J4V1PfVLLuYchC6jBYPxla-eTDC7HTv-A_AJSaDAL4agN7WWLFnc_2tBO0iwg9Jk_wo5FR6X4jNR0zh1sx03UZrwpAKcjTuBSU-LHw-PCuDqYFP4kLVYrlYf_YcFTLZxsiUz88ooqPzGcc8bJwu8r4uCQLkY1GKKWvTjHNCzxBGxyVsGQ1zKSU1-OvOq3nbhECOETk-ygVf8ts.yeYLPLHY0OJ4kDC4vgVSEZbFOgzmBfdWfBjbNyQWbZQ&amp;dib_tag=se&amp;keywords=ladle&amp;qid=1786447405&amp;sprefix=lad%2Caps%2C546&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=cf82ef7c1d7de0ff54f670cf56f4d0b8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C28" r:id="rId27" display="#https://www.amazon.com/ChefAide-Silicone-Ergonomic-Resistant-Nonstick/dp/B0CHGFG64S?crid=QIIJ7VM1WVF&amp;dib=eyJ2IjoiMSJ9.La1iSEcG-MEW7zhzIuKYspMLDGOIUdQbz8_AMVHJWR6O5H1-24U1abeqsNWbV_HkOw1muFOXQF7Op8tasRzOXZPstKcUX7G0QD1OFh_ruoER1AENOSVNEAV6RjffM0DEsJNR9QeF-9RFBt2oeG9ryrLkl2o7KLh4lAWcbI5TiumUA_uW1ZzmjtR3Xz9A8W09CNAJjaKz5dgVezVKPsdvbIYXGDbfjldfF6UP_hi85q4YTaucr9vLQrG_L4nsjn8DRCE-IkZk2nQj-Fbe_U4U9kTpXl8B6P6ik4-VoZmvUXc.xrnbFvPvyzCAPhTbdMbIeaa8kWAlKu4gpm8LrOT9zkI&amp;dib_tag=se&amp;keywords=spatula&amp;qid=1786447434&amp;sprefix=spatula%2Caps%2C651&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=b317254da6af52edf84935b30bb7d093&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C29" r:id="rId28" display="#https://www.amazon.com/Garlic-Press-Easy-Squeeze-Ergonomic-Professional/dp/B07N7KFHVH?crid=TD0OSTRL4FB&amp;dib=eyJ2IjoiMSJ9.DVOWrEMVuQds5c5SVkroV1YHgFVQelKyzAijway-5ucYTxWsVriGLLg_e-LxAcP_gBM_lEV8JsvF5SddukcE1PHfYj9POhIa038OhKz4Z1WmqjS8c1O1wQY0xHSy_gtPPHhH5pE2AObIv0ZrlceFeTU9iQtdydVUiE8_wJEsggMYEuDhsHooWBpDdt-caGUO28wy-UC-SFl3gDvsjplzVcKG4puoGZZ9jMKfTdDz8Kc2Wov3aR7Mxrwjg22cZifcXyCSntrp0rphy9tfgkouFwP0VLjeUyy3UOU1C7hbN0w.-GuJh0wZT6SOvOSgBv5sTZfliJe9JydgXZaXn2HBgYs&amp;dib_tag=se&amp;keywords=garlic%2Bpress&amp;qid=1786447462&amp;sprefix=garlic%2Bpr%2Caps%2C514&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=279de00f5fde249948bc6d3ebd5cbab0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C30" r:id="rId29" display="#https://www.amazon.com/imarku-Japanese-Chef-Knife-Christmas/dp/B01DDBJF12?crid=P1JL5PTKVCSL&amp;dib=eyJ2IjoiMSJ9.ogtZ39PSrD-ERAopQ2MM3VCP_a3dl6ffe6qSY2QaFoOcz8oGUN7M6nxfUCGOkmuTwq3uZILmFIMfI9CKR6HbtdaERpyf8gZneCouzf4ttZr17ulavhgonyJg0S01i2ZJW9_kKnTuQzhzJXZDOIuw8ZebfpvQxb0X36eCZdW_FzupFACVOarwRC93n3S9wJW32TDxpexDdQkXibRkvMrFh73wPGAVexfLgPLRD1J8GnUS2SjRWh2mXWl0k4r7EoC5uyHN9Mn68B3lzNH4u7QcCzrQ9r57yN3o2ClVQiPCcT4.8HLcVWX7WBpQnFO98qmHSZvOO-1enOxBhYwGoXNB3vo&amp;dib_tag=se&amp;keywords=chef%27s%2Bknife&amp;qid=1786447491&amp;sprefix=chef%27s%2Bkni%2Caps%2C559&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=b2350b77530821ac5ff826370713cf5e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C31" r:id="rId30" display="#https://www.amazon.com/Astercook-Deep-Carbonized-Reversible-Charcuterie-Easy-Grip/dp/B0FH6YL3XC?crid=A4FFFNSS5B4Q&amp;dib=eyJ2IjoiMSJ9.vUsBbpa1w7SdehyR5dNno85rMajSPEtI8MRW0HJTGAPIwBRmeRI0F_ekfGI5KJ2B-GHzfWG7FijoG4g8gjeQ1bFsQeYjvrzFMjFI6wX-eQ-fuU2lHrURqC8fhWd04-xo1XhpLaDHF-9gVw3dNZ2oxUJxZ7zUg7BlWkFIbWo7HVxFsrDHtAAK97vygxEEpUyriAgERQMVUsNWJRIuqcrlLpBld5SXozPQEoESjjBiVpsHNc8qHnqac6lSZ32AGEmuELAGNftrToU5o7lz_QpXXPb3PcX3671Z9uBiFaYM2ro.kV-8hceo1PA3PKdjJulr5K0Y4aOwFSNfGKw_8S7h5MM&amp;dib_tag=se&amp;keywords=cutting%2Bboard&amp;qid=1786447530&amp;sprefix=cutting%2Bbo%2Caps%2C509&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=f734b0b1be32e91f76686a1330661035&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C32" r:id="rId31" display="https://www.amazon.com/Elite-Gourmet-ETS623-Grapefruits-Stainless/dp/B0CK9HJ7S2?crid=UKYD8SI8P9CH&amp;dib=eyJ2IjoiMSJ9.1UhghLZQJCJ2KTkTN4ew07Op6NpJGe9jvjxnCv8gsykCvPtHupEbYxeDQNrPBSPFev128ydJ28Fhk55M6H5X67D5HQUM3V1ksBuQEsYWnhFL3FSSnWA_XEl-R89k6REF0ho-Fach8KQfXaOhECJyFIR6ODNVTRp4z_wvMJ1h5O_FY2DFkuMCm9cE5XzL83y4Q4gdtlmlIHg9zEajNhUpYT9ZUrU0lrYSqfuX0qHmeiEP8GRMp3EEGqbuADk0bBWFsoi7_n2i9jMYWb147CT3xGpIQ0ZiBauQX6UJG1iBG8A.ccZbN0L7kXz4HHqG7DCgzA_n_lYouiWMkrmm7sfE7Pk&amp;dib_tag=se&amp;keywords=citrus%2Bjuicer&amp;qid=1786872008&amp;sprefix=citrus%2Bjuicer%2Caps%2C914&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=28affd98ad3bc7313b34443b50536bfb&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C33" r:id="rId32" display="https://www.amazon.com/Spreccio-Mason-Jar-Pitcher-Breastmilk/dp/B0DGCVK1JL?crid=IPKJPEIGAJ58&amp;dib=eyJ2IjoiMSJ9.9l1vM4A3KvgchlohBYfYT5kA329AlVO4aI3BlvpDVf8F7Fg2lBWTZ8SR5rml9CBVBvN3_tedh2s4i7nMpXiM1DX8lBqeMSRgh1JYp8h2tKTcvZifZosHlUbH9TCXAlqmCUcA8yoHVSKl9dbnTLLbZtmcLcxJSFk-wuzbSHYg-XlYQ5vB-FZwQMivn1qpoKp9x1Y4AX4EiCnKdyZ3rCvd9-mCWQJYDh5qd4VCt8wwYzDVzU9_G2ujD0ueeT9qfphpt23C5k1FsC6iQL-ceQHMT7Xk-a81b7xW5lNJ-2GcujM.1ndyCib0tM1CjnH-zB8u6CPXhvMVA-4nVaw6HFwbXV4&amp;dib_tag=se&amp;keywords=glass%2Bpitcher&amp;qid=1786872098&amp;sprefix=glass%2Bpitc%2Caps%2C562&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=266ca3417f7c1e09423feeee72c9750e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C34" r:id="rId33" display="https://www.amazon.com/Immersion-Stainless-Emulsifier-Effortless-Smoothies/dp/B0FSZSKB92?crid=2RYH010QZLP6B&amp;dib=eyJ2IjoiMSJ9.j24smqERTUnUQC9tvuKJTRC1O2DhymNhUTy9LF1ZVEbVaJacQ79Xi_8pSq19SYbhwPzNYMZvNK7_2-hR1CgvdAzXFVjEXuOqtjr_nIF8SoTUdN2ZFMnB6puL49A9LHeq7MzIo-E1YORoVLV932WbPc0ax-B4EPqfVMMvR3-MItykuWUUwZ8q5ljpySZfpN5cwYVLOFcvks6YPYotleo5xm0R92FK7jS4lSk4QuTdatA.SU5DgzcGfKrNJtp4y6rhmsxCbpp4yVbVp0FQ94CTnBQ&amp;dib_tag=se&amp;keywords=immersion%2Bblender&amp;qid=1786872050&amp;sprefix=immersion%2Bblend%2Caps%2C638&amp;sr=8-5&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=ed26bb7454a5ce14f942d75aa542d932&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C35" r:id="rId34" display="https://www.amazon.com/SENSARTE-Nonstick-Stay-cool-Multipurpose-Induction/dp/B09KH38HF2?crid=2VZ5EIV35L5Y2&amp;dib=eyJ2IjoiMSJ9.QAinwdsK-CYNbBOjPxE3HOFR3rVBX2ZDcV0iLx_SGj2bOf61dbGvFbf7xOgRXseTwTkpBQuk8eqRh4s89XEGQRcOJg4pANXzjXdUbEhZYLZrPfpQCpPYG297JuY3p-AdKxyBb9eQdvRnFsCrWmWGJZgBBLKxYyplyktC6IsnXobjKxJFJuGMjbxZkHuuDbdHbzT9UDQ0SwCaSSM9wnicqftri8U6UK14iKtcbWTOHSz9fYIXhMQRr_SxAzS2DIsMdbkj4A06uhfzirBZCCbufEvfDHqdqYBRoYO1HEglG_4.J3YYl_yS9JVkGfPmccm_azx1kN0CkFGP_rP6mvEE3Wc&amp;dib_tag=se&amp;keywords=saucepan&amp;qid=1786872141&amp;sprefix=sauce%2Caps%2C563&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=aac244b2e8e81ae1dbf5b99ffee36dd9&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C36" r:id="rId35" display="https://www.amazon.com/KITESSENSU-Cocktail-Stainless-Bartending-Measuring/dp/B0957GCDKM?crid=SRPXDOA31R27&amp;dib=eyJ2IjoiMSJ9.Myv8qS-yStOlwyOzWRU16SNKJfWP2sc6FLjc4eyuEDu_XBgo-FjsLcMjEzGGNDMkSGSiCh09-6mff24Y1hwz7T-IH82Zf8n26obKPutEFXpd9_9F7KrYnCtKPKtSbfjNQcyCgvLEcMXmr_fanyJ8ZhPedbSoB7kjdtOgStCc0KAGHaqNk9-DXUWRUnYginL8ZDzx4nDn0ZRBlZFsVpM1D4m4A9cX3W1WTdKfuq9ocPMqjn-Ylb3a5_Gz9oq3Ke8H8DFBwkFNV-94vR5WSmS6D55j2ELHgmJxLY0TLW9FsD0.0cvkhzvHgII-P39pQU404pfdnlNJ7_uUId_ydyU--ak&amp;dib_tag=se&amp;keywords=cocktail%2Bshaker&amp;qid=1786872175&amp;sprefix=cocktail%2Bsha%2Caps%2C560&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=9143890d6315842a62c6e211d6613239&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C37" r:id="rId36" display="https://www.amazon.com/NETANY-Overnight-Containers-Airtight-Storage/dp/B0CMQC79L4?crid=7K22MEXBP830&amp;dib=eyJ2IjoiMSJ9.enoJxuZJQnPzeSyAhKOKhlmhdGJFd7oMssDb6ixXe8H2Dbn6iuUnYeAGVN87H1wGX08gIvyNb6J6E__DZ4C_PdtsTSGCZOIhiZ7sqal1fqC83890F7s3RDNDcXBIdbKoqQ8o4H7FeCqJWKXYGcv2FXE-un6bHWFcTzXtcNEJ745Dv9Ij9ZeuitGCTHBNkrkL93wWQsX836J2VdmqNz3flDcM_HhSSoF8l5EtAJnpz68l-OgyYIMGPE1s3WM1KS7s7eBO4tuE_IO6mss10XC7ZfaB8PULTGreKXqwJuJ2rkw.7lwbpo-H72h8eH6zCXwgUVSxEj2yBFDJRsRGtJcFDN4&amp;dib_tag=se&amp;keywords=freezer-safe%2Bjars&amp;qid=1786872212&amp;sprefix=freezer-safe%2Bja%2Caps%2C557&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=697fd55ab6f7fbf6975059c5d21b8495&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C38" r:id="rId37" display="https://www.amazon.com/Joyoldelf-Heavy-Stainless-Potato-Masher/dp/B014499LUW?content-id=amzn1.sym.b7a3dce9-da16-4d10-a59e-2752928fe1a8%3Aamzn1.sym.b7a3dce9-da16-4d10-a59e-2752928fe1a8&amp;crid=1C7RUBC175C5U&amp;cv_ct_cx=potato%2Bmasher&amp;keywords=potato%2Bmasher&amp;pd_rd_i=B014499LUW&amp;pd_rd_r=9b7d5c3a-dfe4-4797-91f7-bb533185f137&amp;pd_rd_w=sVUKc&amp;pd_rd_wg=r7M6B&amp;pf_rd_p=b7a3dce9-da16-4d10-a59e-2752928fe1a8&amp;pf_rd_r=2508QYV67H1VQXX6H0YJ&amp;qid=1786872246&amp;sbo=RZvfv%2F%2FHxDF%2BO5021pAnSA%3D%3D&amp;sprefix=potato%2Bmashe%2Caps%2C589&amp;sr=1-2-925d4041-2745-4edd-b995-62e9e595df4e-spons&amp;aref=lQwm73e8i5&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9zZWFyY2hfdGhlbWF0aWM&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=8ca4353da3c88432096e0cd05e5ea10b&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
-    <hyperlink ref="C39" r:id="rId38" display="https://www.amazon.com/Multipurpose-Strainer-Nonstick-Effortless-Dishwasher/dp/B071L32Q8W?crid=18P0O4OLX9ITW&amp;dib=eyJ2IjoiMSJ9.Hk5FM9ts2t-lgjKM6c-bIuFz37EC2J1UQkHWsRJuDs8mQNkC0IMrQm0FrFPLMKDnfEwK_-xVbq9oIPyHoG4teGyr9KgWZTUbHnrne8F11WePQkI_Kf24uwjErshzpoHx6vB3vbsT4V6vBfv-236Hhkw9hov1O96AUc4Hlo_ek5x3_xVJhNZE9ds1zTRlgEWhgd4Kf1b9eHPpVbhuOf-rd-9oGM98GVv25hBgc5DXU_aDdimxYMLNzDLZ5NZAeseqXP4qeRvMrbxx4vWBYsjgxt6DsjVkYJQmdxo-DwsuuVc.5LJ4LmQtuB3e_KCQxdQRwBZ-rZo7TklJPqTR3hA1WFY&amp;dib_tag=se&amp;keywords=stockpot&amp;qid=1786872288&amp;sprefix=stock%2Caps%2C555&amp;sr=8-2&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=3c345bda2c468c8f0c4e7ebd53896fcb&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C40" r:id="rId1" display="https://www.amazon.com/TurboBlaze-Premium-Ceramic-Coating-90%C2%B0-450%C2%B0F/dp/B0C33CHG99?crid=29K174U7RQHED&amp;dib=eyJ2IjoiMSJ9.JvIQTiQYIa-7vH5--3jg964Nf0p9WdZAK-1rFngdE1qGM52kKAeYw9Spp1PcLbq2qNDAfw3uEx2H6W-EFkqsdxLXGnACw1V8E1qj9ygR4ltV8I7ae4AVnWNULiWAQn0XzCG3wxdpH4V3GpRQyA_duvD4pgTzx87lPL7Bi3RZ_Zv8qmydNpS3h2S9xcyOTN3Q7L0NxnhsP1zMshbUKW9-389sbsvxO8ivjkVLFTywoNY.x8J6j-z5dUwMipVngmAM2ij0iXUm61IpGmkBkKphkoU&amp;dib_tag=se&amp;keywords=air%2Bfryer&amp;qid=1787294833&amp;sprefix=air%2Bfr%2Caps%2C587&amp;sr=8-4&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1201615d33fb8c566ab906e6a65cd11d&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C41" r:id="rId2" display="https://www.amazon.com/Rubbermaid-Brilliance-Airtight-Container-BPA-Free/dp/B0752ZJ5LF?crid=Z0F89GGNT4UY&amp;dib=eyJ2IjoiMSJ9.5MRpyVweaPJP07XGqOBD1wsdmjhYMozLz6iXZz6aQWKYymueUSn82sJng_h6kVUZXe2WRHNRJTeVmfKQtgDUTT9GUKFVhjtniql21svT65gOVYaRHD15jDuzJh44Odpsz4D_qXvisfcJdjlhSPtJ2QH9f4o_I9l9MKA81HbEsYlaKAPx_TJmO2dY4n4oh155BIg45OGtNH1ligNedn0njlf--CK9VfN5_HJDRq8ik-G61pzopxg2a9vuuTH3t-vVpZ21D3Kf78X10JCuxcrz1bKNUsQH0gZ8d_6ytiGhY_Y.f9Nd8K9YN_4AuKc3xiCT9lEmMtQ-1a8gKo0a8Dwtm0s&amp;dib_tag=se&amp;keywords=airtight%2Bcontainer&amp;qid=1787294895&amp;sprefix=airtight%2Bconta%2Caps%2C557&amp;sr=8-19&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1a4abfd6227ead40175359daf590e743&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C42" r:id="rId3" display="https://www.amazon.com/Cuisinart-CISB-111-Smashed-Burger-Press/dp/B07SZFHKVZ?crid=1IINFDVVYUJDM&amp;dib=eyJ2IjoiMSJ9.2HjCnozck-eoA00aOrjZesor3pCxus5hokq_4DlRPX4EnP6X1qF_V1fGRoaDGLWugk2N3z5YgQ4Y90253AUxfGHNXo2fSBW7zGJin2tRRwy457b1uzXsD2C6PzznhUdcrbEMlJJHTznVIreGy6Q4JGk_w-c6P_YoffVoOa3Q9TQM7jFnCBQkCJtaleh4OfgrW2CrDB49-fcwocVvX7JffiVbTe4RUbmjQ1xHPLciGZ4.v-APOZeiC_xO-YKvTb-XZdOv-Tag0mK_VV_Af7E_LAI&amp;dib_tag=se&amp;keywords=burger%2Bpress&amp;qid=1787294991&amp;sprefix=burger%2Bpr%2Caps%2C532&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=b5cec603147e56eec4c3073c54a1a1f1&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C43" r:id="rId4" display="https://www.amazon.com/Elite-Gourmet-ETS623-Grapefruits-Stainless/dp/B0CK9HJ7S2?crid=1YIQ27RXITQET&amp;dib=eyJ2IjoiMSJ9.MpofArt3UHaOnw_l4i2df38sTpxWZ2mm06nPKPRR6OM2tjaJKIvl9z7PW9TMde0bcK2LitegnDPKYwl_I9BNQzMLS5GTN5vkyyySMpSPRuf-WaVd3aHJIhxMcUo8kwfCWS6WqbjnbAmp-n_dHNP78PgaSUo0E5RTbi2OkFthR-YdJWhIRHBJx1ooKQMAt2XShRtb09VpZ1uWKw2gpjELCaFIMQ2WsE5hP7z9oDgGNDeHgkaZ32RtFb4R-5_IVumTkWFi1jkzuQiInSM7nEL0GiChFPNvlPQtQv2FfT_NuMg.icwAVliH5Ko-4s-E3V8fmVP9v9JZa6gWGcrFzqHvL8c&amp;dib_tag=se&amp;keywords=citrus%2Bsqueezer&amp;qid=1787295033&amp;sprefix=citrus%2Bsquee%2Caps%2C589&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=263283c6248f72d5cc927a2ce4d403b4&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C44" r:id="rId5" display="https://www.amazon.com/ChefAide-Silicone-Ergonomic-Resistant-Nonstick/dp/B0CHGFG64S?crid=2A0SVC5HLZVJ1&amp;dib=eyJ2IjoiMSJ9.-rDpl5_Q4Gx78sf1baalWfpcVTZ7P4zGKH2CIIZvnR423EnItEOMbYiaGhkNPGk3fgCdca9ZnGU_BGN7ly2ItFTK2iM6-uL_AmRvHg1wdBMK5a_H2wISQnSSJbaQ0XFlHW5zev5ToeM8ChQZ9z_YvG1SdDEux6qsbJZsK99s6ByZ65VFsUQS3rPlVU7ubp8odf9uDhya2YmttiYzhUsjbQLVlVdYV_L0xLQOZAGOaDO88KrZiI1GCxTwOG4uum4uLoHwPkyP6jcWcCMa2wOAyyOFCp9GAsUSEuH8TwnoFf0.2Ya68W0VD7Rb3p8-9x7Et4cNA8ZgnokckXwyHfi3c2w&amp;dib_tag=se&amp;keywords=flexible%2Bspatula&amp;qid=1787295074&amp;sprefix=flexible%2Bspa%2Caps%2C567&amp;sr=8-9&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=7ed999d8d8e27438d02797241c24afc6&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C45" r:id="rId6" display="https://www.amazon.com/Containers-Airtight-Leak-Proof-Microwave-Dishwasher/dp/B0DPJXW27G?crid=1CWVOGTYQYQ8Y&amp;dib=eyJ2IjoiMSJ9.ybs2wvTHoEH1p_vOKWw5BqHKflEJSlHogAZnV8P9w0UlCVIcbCLyeUJgxs4O3DCch-qu2f1tlq4MSRY_DIvvG_PdUlDCRvqTzjPcfbRa5c0Yw4yftAloxYMFkeRQZmZsaKYMS5GAr64RkYG-_5k7yzLOlYrjC3y3YbdYH_oJcLR-f-Bnzla80vE2l_XxgHhikQRmw7vkv1oub1w1fRnUvb68lKrMar5s8EHBgEL9oLVZgwua7y37zqWQ5jJrNOt25QlV6YMUtD8_JoAPwEUfHKDWYAFshngyYm0tD7KObcs.-ZtLxlyrwuMbqoRkWwOJeGKQdIwSQeb-TH3H94Xqff8&amp;dib_tag=se&amp;keywords=glass%2Bmeal%2Bprep%2Bbowls&amp;qid=1787295119&amp;sprefix=glass%2Bmeal%2Bprep%2Bbowls%2Caps%2C575&amp;sr=8-17&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=caf1539ee1a93341975fa80c9507a3c0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C46" r:id="rId7" display="https://www.amazon.com/UTEBIT-Infuser-Insulated-Camping-Outdoor/dp/B0BR8SK56M?crid=33E7HR6O2HEPS&amp;dib=eyJ2IjoiMSJ9.y0PuPqw2grQkyLWqPgX_mQYsZ6vgR29h7ATgfAICQ-4Eszad_vgAGq-QZdGodPpoqiFEbyX_yd8CW-kOGnalTRLMvQBo5_DMFNXM5Ex1F6ERPPD0V6jJox-PW8cb0AOFHVCD8-552s5cQPRpsk7V_vwIgP4gr7f1dhUhT8mhxGoFRRVfM7BqrLTZsoxqo7weDbRR6fbGflbxdDVnC5nesSNbGIlVyJYKD_3C-xMmt1NDKjmZS1Lwe7AEDU_w0-wVt-BVEohQg401otSAgLIRtw0IbvJVBlGrhNWwdroelsI._k7QkHSbFAj85G9ckqAbOnrxWY32L4s13URp_8VgYcs&amp;dib_tag=se&amp;keywords=infuser%2Bwater%2Bbottle&amp;qid=1787295196&amp;sprefix=infuser%2Bwater%2Bbott%2Caps%2C533&amp;sr=8-5&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=c02dfdc05b9ed8e0cc5d5ce1e4d89838&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C47" r:id="rId8" display="https://www.amazon.com/Thermometer-Cooking-BACKLIGHT-WATERPROOF-Temperature/dp/B00S93EQUK?crid=2V45R8BOOGT2&amp;dib=eyJ2IjoiMSJ9.8Ger4dMy4c3dRylJ0ztFU3EMn17qargrZcTgRn6jMofvVZEAm0qcJ_VRE-2yUvgB4kicBhPr6QahzAhlE7EE9jPOtHsl1f7yZ3Qb5xcHVJ7ZWr5LvdSVRs4didU44e4BGd-ksJU1vNB7ieK7_4OAfNKukB2U_dIzt1A9hzOhIxBjXTjRDGsUZbvg315ak52dce9iXOajFRd9szjVKAv3pPAVrkH5dLhEnAk8XoyOgJuQG6pKRD07iOjR0ioY_vq2EWvCCud2q1gRMFFopSiTg6VvAi8NTf4368O1XYdLQXc.dv3EBSg01A8M-FRJVdXg58QbiKduIEOoz2gmOzndzGs&amp;dib_tag=se&amp;keywords=instant+read+thermometer&amp;qid=1787295246&amp;sprefix=instant+read+thermo%2Caps%2C605&amp;sr=8-7&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=ccaf292f3bc1f53792e628b2f803223e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C48" r:id="rId9" display="https://www.amazon.com/WEPSEN-Stainless-Kitchen-Measuring-Prepping/dp/B0CT2NWXX8?content-id=amzn1.sym.29113e31-4f10-4131-ad60-91d41893b2fc%3Aamzn1.sym.29113e31-4f10-4131-ad60-91d41893b2fc&amp;crid=2PGTJ1KK0JV9E&amp;cv_ct_cx=large%2Bmixing%2Bbowl&amp;keywords=large%2Bmixing%2Bbowl&amp;pd_rd_i=B0CT2NWXX8&amp;pd_rd_r=9195d263-901a-4a9d-92a3-5b5b3c93cbb7&amp;pd_rd_w=uIsjq&amp;pd_rd_wg=3C3Ql&amp;pf_rd_p=29113e31-4f10-4131-ad60-91d41893b2fc&amp;pf_rd_r=1MM32EDSCWCZG5X1TCPG&amp;qid=1787295282&amp;sbo=9ZOMT9Jm0JH%2Ft%2BWi68iDSA%3D%3D&amp;sprefix=large%2Bmixing%2Bbow%2Caps%2C553&amp;sr=1-3-f7d8a1b7-d68f-4a86-bfcb-111c62272989-spons&amp;aref=uR0PevFOnJ&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9zZWFyY2hfdGhlbWF0aWM&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=c5a096620ca09998f1199d8e01b134ab&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C49" r:id="rId10" display="https://www.amazon.com/Ball-Mouth-Mason-mason-Bands/dp/B097HTTNF3?crid=3EQ9W7GFM88NE&amp;dib=eyJ2IjoiMSJ9.lqj6Tzyfa-gcoNR1ERjIOYDT4frKh5IBawXIFyXnuydFyQqclrZBgW3OTNVjx9O9j6aYm06mRCgqHP5uS0UH6WVLV-7T3ah1O7TrqB_QDGYK1beIAUa8OvRjn8mt7FQ0gmnOIephoHXFnBo3AfNOIkTuDLgex9-XiNZ7DSpeUcYS6ycTtw2ROA4AFA2P5mQLsWvRGkHCfrkVQBXpt2zuiCNyYgEFa8Ev_9iWmLcDwrgTc2y6E-OZYxfVJlaWxZsVxxMBtwJEwqPriFVN3NCXsF3v-4oJGQ9holnbFR2dvZ0.ecf5ioiuMD1yPkTKbtsDFgosao1gsILrA7Sdq4ge9cQ&amp;dib_tag=se&amp;keywords=mason%2Bjars&amp;qid=1787295330&amp;sprefix=mason%2Bja%2Caps%2C589&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=f9026d2a5d2910079203befae79daf54&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C50" r:id="rId11" display="https://www.amazon.com/KitchenAid-KO119OHOBA-Gourmet-Tenderizer-9-45-Inch/dp/B07Q2WVG1Z?crid=38F4NQV8WDJOD&amp;dib=eyJ2IjoiMSJ9.k8Nt-b8zXr54n7L4-B4CKXAYf1FWHcwCUdjEv52YlIB2qJ3rh0z_xF719kyUxBjrOu4iFdAOZuKtoKDJzrAt8p0TclHqxQljGXjmwvmKQ2PTY_dEGuyvOShPGAup3mF_RyY89ydXyQNg3wjPZwiOUMmsT436OrhtH1LAhklyjAHsaZZ3D1RVbybQug6AUz020lImdzHczmZ17Uj7yyswn4gL9LukFRsbrWqBoOKd1OkW39xsh_zukHMRGJ5KsZeR5HMx9LOOm2u4jwAp-abdCEQcO2PNW5xmWuE3B7EFp6w.TbAuD567rEFWoPt_9qCXm5fE7Us8xYEd8SgvekViDYY&amp;dib_tag=se&amp;keywords=meat%2Bmallet&amp;qid=1787295368&amp;sprefix=meat%2Bmallet%2Caps%2C555&amp;sr=8-8&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=d2a147638fa7aabdf0f4e00752440447&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C51" r:id="rId12" display="https://www.amazon.com/Lodge-Skillet-Pre-Seasoned-Ready-Stove/dp/B00006JSUA?crid=3AZT7NZUHRXBD&amp;dib=eyJ2IjoiMSJ9.KAwBSzSJL8L5NQvLjg83Wg4GkPnKsr5AbNi7kiAMn7zzmOAiELpFOh_dQKvCaTamh0-ClyzLuBkeqrQOdOo1RzY_Tv8JmCIL7uVB2vIIIADAM-bmDuAZUN748UDBeJDLbQHTk8ZqKvoPJl7vjarAlt1nstLYQqgth4CpWPKKGEUAznf4I9eefj58hqV_IbUY3h440imhMzzfHrDyuK18i0NuQdicqVIjTSFABkhcv14ooNcsvgJwr-VqnEAnXOuQ3Ik3jIR3BnAODTY9VEktNxVMShEhLQG27ulnxeKH6V0.KWHN3bnxg6zo2lXz_5VWpd6XceMfXAqmNiu28FGp0v4&amp;dib_tag=se&amp;keywords=oven%2Bsafe%2Bskillet&amp;qid=1787295409&amp;sprefix=oven%2Bsafe%2Bskill%2Caps%2C581&amp;sr=8-6&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=5abda6359e88e1a32c81cde06bbb4b2f&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C52" r:id="rId13" display="https://www.amazon.com/HOTEC-Silicone-Resistant-Marinades-Dishwasher/dp/B09JNRZHRT?crid=IHGMIQ13RZ2R&amp;dib=eyJ2IjoiMSJ9.9PjoV_tUr5meI1KqtWNrWerj8iQYjaQUGDa1Q5z_1bBUqLA5vNaKD0Cd6N0uSrjIHq70Nxh90KFbNejI-VdvVeHuTq5Xip673_usxYz7nGpa6TYUgA1lsxMlS7AxpXDayCJ7x11mCutpUs-gXkt3eWCixf8w87_urNTxy58d9UA9DyfUmnHu9kvAkkf6lyY4dUAvtEJxP9J1OHGNKA9OVWY4-5uCI5RJ7GjVGMOsMmbj6Y3tmIy_01yhW2fLzpaiV-3NAb86ogBESTe2JWh0w8hTEyF4Th3L7ePJPv9Zd4o.wCCOBz8XAme674vClvmAT7zvnG1Asr6iopICDPKNnNI&amp;dib_tag=se&amp;keywords=pastry%2Bbrush&amp;qid=1787295453&amp;sprefix=pastry%2Bbrush%2Caps%2C579&amp;sr=8-9&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=1a7a90fc0085edb0f8ba1813f16049fe&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C53" r:id="rId14" display="https://www.amazon.com/ComSaf-Mini-Mason-Jars-4oz/dp/B09YRC9SXW?crid=CVHMLQUIH3FS&amp;dib=eyJ2IjoiMSJ9.6_G97mRQ6FsY74JoSCi-A4aYxpMtF9d6g81RQJdwj6UT9NdkqRjc2gJwVwQWVfPvV8XRux1JP4y9kwqa2ADx1w6VjBJ23LxbqTO7k0Obn0ybegP8zUjw0PrqYTVVvUp2a0ajUcti5I5JWimD1GyBnRv4uJMWHlwXZAJpl9IXHK1-Uw0bUko3KophDmYCt_NYZfZfqGOPDWlFbLTq5FdxW8VlUD1iO2Ssc3teq5Rz11spwrkj3SEG1wAZo1a602wKdl3mDCRA4v75uRoRs_L_-8OWXwhwXW2uBf8VkFQFVNE.SuvHK5fSC7xzDx0Wfrah1wVW6ZxEsIbyOYL2BbmApUk&amp;dib_tag=se&amp;keywords=small%2Bmason%2Bjars&amp;qid=1787295494&amp;sprefix=small%2Bmason%2Bja%2Caps%2C592&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=6312b0bb70fc760ae595d1739f0611b0&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C54" r:id="rId15" display="https://www.amazon.com/Cuisinart-719-16-Classic-Stainless-Saucepan/dp/B00008CM69?crid=3MDFOTS2HUROE&amp;dib=eyJ2IjoiMSJ9.QAinwdsK-CYNbBOjPxE3HMPr4hxU2ZhD8wbPZ1y-jiCtW_J1TbyOKBy1uxlp56ycFrfLdtWIV8XgIxRd-MKRPrnUi-rvJ9Wtrsbg_9oaYcmdaQLbPX-3rH9Zzz1WKYrYovhgiJjcIEnaEzQsRXExt5aIpewu97jUtL0_fBXfvMl-vbBv77V6r6-ZI4BlnSWaxXQ2VOHWuSgE4Ph51XRTBxVeym_JZ9k0bJMHJG9XeC6FR8TFN3-t4Jpa157YCOU6CV3d4dwgrNrmovn4d0leB44Xiu7Ojs1Q-NKkmaRyCz8.r1s79ymMmqskg66Gaphq_82T-VW6qdruYBAsp9lKE9U&amp;dib_tag=se&amp;keywords=small%2Bsaucepan&amp;qid=1787295530&amp;sprefix=small%2Bsaucep%2Caps%2C551&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=03169d89cccb51075cc93718a03703b8&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C55" r:id="rId16" display="https://www.amazon.com/NileHome-Stainless-Whisking-Blending-Stirring-3/dp/B08SWBRTRK?crid=2SJCTGODY5ZTU&amp;dib=eyJ2IjoiMSJ9.9CbAVoJJ-Ip6yMNfWgFmaof9D1Rwh3PRS-hkzkoUO9UXyEi9aGNZfLqk38yttMH_gIM_pMu8rsQ3OqTX7Cz7b_4kY7e8p3TFRtzWIdmG9GB1EMuudgmX2-6Ta309ttVykeG5Gs7dD7B1cCFczjB2aM2HR6_fsvADbLSDBsU_PvB2wwj2MrjPe0g8qylrB3SV8bM_Z0RbQucRWzTtDUz3DZeH53K1f2Jq0Dq8xjjOwhVwj_YVrBiuFUBM7ZGkhyRN9BJPZA57d_mS7IHrbq36EDPecT3TlnwC8W0N8q3-f_s.LVwHcWq_WHK8mpgK_WNOW6vzASnGRE_SIIWMAgo9bfU&amp;dib_tag=se&amp;keywords=small%2Bwhisk&amp;qid=1787295573&amp;sprefix=small%2Bwhis%2Caps%2C595&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=ee49d14fa45547d3cbcada6d43130b5e&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
+    <hyperlink ref="C56" r:id="rId17" display="https://www.amazon.com/Drinking-Water-Crystal-Highball-Glasses/dp/B0DBL3WXYW?crid=3SDY3XAS1V3MU&amp;dib=eyJ2IjoiMSJ9.BruIBv41Cv5aVUrTFtq9KMMI_9pmyL-lJexIBGaQIQ6Nnnn46SlOV83fWHS5y-GEcT8BmfmCVOK-AJG9y9EtoGoLnZYxLB47GqrClAXiGuZoWbai6TJrjVKdjh4zCS5Q7ApeIc2_pwyb9EEqb79JxPtoDfsM4J4mpq7JG_w7yHo6_zJQPGGJ376cBjmAgFDRqF6C8KaIK_a8tLNkKLkf9qIeEafSuXlaVSqzsDyL2qOZBSQvKE3CoGOuHL4ps249H73ucMKJOv2iIWfKMDg4zh86imqfoTp3A_IUZTtjON8.0fQIsdvGGjfSPxZoE1fo31xzH1LgOEqHuGeBZscqLSs&amp;dib_tag=se&amp;keywords=tall%2Bglasses&amp;qid=1787295615&amp;sprefix=tall%2Bglas%2Caps%2C554&amp;sr=8-7&amp;th=1&amp;linkCode=ll2&amp;tag=theorgani0014-20&amp;linkId=0ae6d191a7d037f96e6bede877489fe2&amp;language=en_US&amp;gaOptInStatus=true&amp;ref_=as_li_ss_tl"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -1372,61 +1600,50 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="80"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>109</v>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>